<commit_message>
Add radii of gyration to tension member calculations for single angles
Updates the Angle Properties Table.xlsx and pages/1_Tension_Members.py to include rx, ry, and rz radii of gyration for single angles, improving the accuracy of tension member calculations. Also displays rx and ry for double angles, WT tees, and channels.

Replit-Commit-Author: Agent
Replit-Commit-Session-Id: ad543291-9022-4756-a3ba-a22eaaae8ef0
Replit-Commit-Checkpoint-Type: full_checkpoint
Replit-Commit-Event-Id: 4bedf91a-bee5-4b1b-92d1-c03b11e8026e
Replit-Commit-Screenshot-Url: https://storage.googleapis.com/screenshot-production-us-central1/bda54d3c-93de-4e83-8aea-5228fc4f95b1/ad543291-9022-4756-a3ba-a22eaaae8ef0/USKjceE
Replit-Helium-Checkpoint-Created: true
</commit_message>
<xml_diff>
--- a/data/Angle Properties Table.xlsx
+++ b/data/Angle Properties Table.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E150"/>
+  <dimension ref="A1:H150"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -442,6 +442,21 @@
           <t>Area (mm2)</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>rx (mm)</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>ry (mm)</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>rz (mm)</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -461,6 +476,15 @@
       <c r="E2" t="n">
         <v>15100</v>
       </c>
+      <c r="F2" t="n">
+        <v>77.30000000000001</v>
+      </c>
+      <c r="G2" t="n">
+        <v>77.30000000000001</v>
+      </c>
+      <c r="H2" t="n">
+        <v>49.7</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -480,6 +504,15 @@
       <c r="E3" t="n">
         <v>13700</v>
       </c>
+      <c r="F3" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="G3" t="n">
+        <v>77.7</v>
+      </c>
+      <c r="H3" t="n">
+        <v>49.8</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -499,6 +532,15 @@
       <c r="E4" t="n">
         <v>12300</v>
       </c>
+      <c r="F4" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="G4" t="n">
+        <v>78.2</v>
+      </c>
+      <c r="H4" t="n">
+        <v>49.9</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -518,6 +560,15 @@
       <c r="E5" t="n">
         <v>10800</v>
       </c>
+      <c r="F5" t="n">
+        <v>78.60000000000001</v>
+      </c>
+      <c r="G5" t="n">
+        <v>78.60000000000001</v>
+      </c>
+      <c r="H5" t="n">
+        <v>50.1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -537,6 +588,15 @@
       <c r="E6" t="n">
         <v>9340</v>
       </c>
+      <c r="F6" t="n">
+        <v>79.10000000000001</v>
+      </c>
+      <c r="G6" t="n">
+        <v>79.10000000000001</v>
+      </c>
+      <c r="H6" t="n">
+        <v>50.3</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -556,6 +616,15 @@
       <c r="E7" t="n">
         <v>10800</v>
       </c>
+      <c r="F7" t="n">
+        <v>61.40000000000001</v>
+      </c>
+      <c r="G7" t="n">
+        <v>61.40000000000001</v>
+      </c>
+      <c r="H7" t="n">
+        <v>39.6</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -575,6 +644,15 @@
       <c r="E8" t="n">
         <v>9670</v>
       </c>
+      <c r="F8" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="G8" t="n">
+        <v>61.8</v>
+      </c>
+      <c r="H8" t="n">
+        <v>39.7</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -594,6 +672,15 @@
       <c r="E9" t="n">
         <v>8520</v>
       </c>
+      <c r="F9" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="G9" t="n">
+        <v>62.2</v>
+      </c>
+      <c r="H9" t="n">
+        <v>39.8</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -613,6 +700,15 @@
       <c r="E10" t="n">
         <v>7350</v>
       </c>
+      <c r="F10" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="G10" t="n">
+        <v>62.7</v>
+      </c>
+      <c r="H10" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -632,6 +728,15 @@
       <c r="E11" t="n">
         <v>6200</v>
       </c>
+      <c r="F11" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="G11" t="n">
+        <v>63.1</v>
+      </c>
+      <c r="H11" t="n">
+        <v>40.1</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -651,6 +756,15 @@
       <c r="E12" t="n">
         <v>5600</v>
       </c>
+      <c r="F12" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="G12" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="H12" t="n">
+        <v>40.2</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -670,6 +784,15 @@
       <c r="E13" t="n">
         <v>4990</v>
       </c>
+      <c r="F13" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="G13" t="n">
+        <v>63.6</v>
+      </c>
+      <c r="H13" t="n">
+        <v>40.3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -689,6 +812,15 @@
       <c r="E14" t="n">
         <v>8370</v>
       </c>
+      <c r="F14" t="n">
+        <v>63.3</v>
+      </c>
+      <c r="G14" t="n">
+        <v>43.7</v>
+      </c>
+      <c r="H14" t="n">
+        <v>32.4</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -708,6 +840,15 @@
       <c r="E15" t="n">
         <v>7390</v>
       </c>
+      <c r="F15" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="G15" t="n">
+        <v>44.1</v>
+      </c>
+      <c r="H15" t="n">
+        <v>32.5</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -727,6 +868,15 @@
       <c r="E16" t="n">
         <v>6380</v>
       </c>
+      <c r="F16" t="n">
+        <v>64.10000000000001</v>
+      </c>
+      <c r="G16" t="n">
+        <v>44.5</v>
+      </c>
+      <c r="H16" t="n">
+        <v>32.6</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -746,6 +896,15 @@
       <c r="E17" t="n">
         <v>5390</v>
       </c>
+      <c r="F17" t="n">
+        <v>64.60000000000001</v>
+      </c>
+      <c r="G17" t="n">
+        <v>44.90000000000001</v>
+      </c>
+      <c r="H17" t="n">
+        <v>32.8</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -765,6 +924,15 @@
       <c r="E18" t="n">
         <v>4870</v>
       </c>
+      <c r="F18" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="G18" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="H18" t="n">
+        <v>32.9</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -784,6 +952,15 @@
       <c r="E19" t="n">
         <v>4350</v>
       </c>
+      <c r="F19" t="n">
+        <v>65</v>
+      </c>
+      <c r="G19" t="n">
+        <v>45.40000000000001</v>
+      </c>
+      <c r="H19" t="n">
+        <v>33</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -803,6 +980,15 @@
       <c r="E20" t="n">
         <v>3820</v>
       </c>
+      <c r="F20" t="n">
+        <v>65.3</v>
+      </c>
+      <c r="G20" t="n">
+        <v>45.6</v>
+      </c>
+      <c r="H20" t="n">
+        <v>33.1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -822,6 +1008,15 @@
       <c r="E21" t="n">
         <v>7100</v>
       </c>
+      <c r="F21" t="n">
+        <v>63.8</v>
+      </c>
+      <c r="G21" t="n">
+        <v>26.3</v>
+      </c>
+      <c r="H21" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -841,6 +1036,15 @@
       <c r="E22" t="n">
         <v>6280</v>
       </c>
+      <c r="F22" t="n">
+        <v>64.3</v>
+      </c>
+      <c r="G22" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="H22" t="n">
+        <v>21.6</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -860,6 +1064,15 @@
       <c r="E23" t="n">
         <v>5430</v>
       </c>
+      <c r="F23" t="n">
+        <v>64.7</v>
+      </c>
+      <c r="G23" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="H23" t="n">
+        <v>21.7</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -879,6 +1092,15 @@
       <c r="E24" t="n">
         <v>4600</v>
       </c>
+      <c r="F24" t="n">
+        <v>65.2</v>
+      </c>
+      <c r="G24" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="H24" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -898,6 +1120,15 @@
       <c r="E25" t="n">
         <v>4160</v>
       </c>
+      <c r="F25" t="n">
+        <v>65.40000000000001</v>
+      </c>
+      <c r="G25" t="n">
+        <v>27.4</v>
+      </c>
+      <c r="H25" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -917,6 +1148,15 @@
       <c r="E26" t="n">
         <v>3710</v>
       </c>
+      <c r="F26" t="n">
+        <v>65.7</v>
+      </c>
+      <c r="G26" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="H26" t="n">
+        <v>22.1</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -936,6 +1176,15 @@
       <c r="E27" t="n">
         <v>3260</v>
       </c>
+      <c r="F27" t="n">
+        <v>65.90000000000001</v>
+      </c>
+      <c r="G27" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="H27" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -955,6 +1204,15 @@
       <c r="E28" t="n">
         <v>4960</v>
       </c>
+      <c r="F28" t="n">
+        <v>56.40000000000001</v>
+      </c>
+      <c r="G28" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="H28" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -974,6 +1232,15 @@
       <c r="E29" t="n">
         <v>4200</v>
       </c>
+      <c r="F29" t="n">
+        <v>56.8</v>
+      </c>
+      <c r="G29" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="H29" t="n">
+        <v>22.1</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -993,6 +1260,15 @@
       <c r="E30" t="n">
         <v>3390</v>
       </c>
+      <c r="F30" t="n">
+        <v>57.3</v>
+      </c>
+      <c r="G30" t="n">
+        <v>28.5</v>
+      </c>
+      <c r="H30" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1012,6 +1288,15 @@
       <c r="E31" t="n">
         <v>2980</v>
       </c>
+      <c r="F31" t="n">
+        <v>57.5</v>
+      </c>
+      <c r="G31" t="n">
+        <v>28.7</v>
+      </c>
+      <c r="H31" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1031,6 +1316,15 @@
       <c r="E32" t="n">
         <v>2580</v>
       </c>
+      <c r="F32" t="n">
+        <v>57.8</v>
+      </c>
+      <c r="G32" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="H32" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1050,6 +1344,15 @@
       <c r="E33" t="n">
         <v>7080</v>
       </c>
+      <c r="F33" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="G33" t="n">
+        <v>45.5</v>
+      </c>
+      <c r="H33" t="n">
+        <v>29.6</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1069,6 +1372,15 @@
       <c r="E34" t="n">
         <v>6260</v>
       </c>
+      <c r="F34" t="n">
+        <v>45.90000000000001</v>
+      </c>
+      <c r="G34" t="n">
+        <v>45.90000000000001</v>
+      </c>
+      <c r="H34" t="n">
+        <v>29.6</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1088,6 +1400,15 @@
       <c r="E35" t="n">
         <v>5420</v>
       </c>
+      <c r="F35" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="G35" t="n">
+        <v>46.3</v>
+      </c>
+      <c r="H35" t="n">
+        <v>29.7</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1107,6 +1428,15 @@
       <c r="E36" t="n">
         <v>4580</v>
       </c>
+      <c r="F36" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="G36" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="H36" t="n">
+        <v>29.8</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1126,6 +1456,15 @@
       <c r="E37" t="n">
         <v>4140</v>
       </c>
+      <c r="F37" t="n">
+        <v>46.90000000000001</v>
+      </c>
+      <c r="G37" t="n">
+        <v>46.90000000000001</v>
+      </c>
+      <c r="H37" t="n">
+        <v>29.9</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1145,6 +1484,15 @@
       <c r="E38" t="n">
         <v>3700</v>
       </c>
+      <c r="F38" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="G38" t="n">
+        <v>47.1</v>
+      </c>
+      <c r="H38" t="n">
+        <v>30</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1164,6 +1512,15 @@
       <c r="E39" t="n">
         <v>3250</v>
       </c>
+      <c r="F39" t="n">
+        <v>47.40000000000001</v>
+      </c>
+      <c r="G39" t="n">
+        <v>47.40000000000001</v>
+      </c>
+      <c r="H39" t="n">
+        <v>30.1</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1183,6 +1540,15 @@
       <c r="E40" t="n">
         <v>2810</v>
       </c>
+      <c r="F40" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="G40" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="H40" t="n">
+        <v>30.2</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1202,6 +1568,15 @@
       <c r="E41" t="n">
         <v>2350</v>
       </c>
+      <c r="F41" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="G41" t="n">
+        <v>47.8</v>
+      </c>
+      <c r="H41" t="n">
+        <v>30.3</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1221,6 +1596,15 @@
       <c r="E42" t="n">
         <v>5150</v>
       </c>
+      <c r="F42" t="n">
+        <v>47.2</v>
+      </c>
+      <c r="G42" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="H42" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1240,6 +1624,15 @@
       <c r="E43" t="n">
         <v>4470</v>
       </c>
+      <c r="F43" t="n">
+        <v>47.6</v>
+      </c>
+      <c r="G43" t="n">
+        <v>28.6</v>
+      </c>
+      <c r="H43" t="n">
+        <v>21.9</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1259,6 +1652,15 @@
       <c r="E44" t="n">
         <v>3790</v>
       </c>
+      <c r="F44" t="n">
+        <v>48</v>
+      </c>
+      <c r="G44" t="n">
+        <v>28.9</v>
+      </c>
+      <c r="H44" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1278,6 +1680,15 @@
       <c r="E45" t="n">
         <v>3430</v>
       </c>
+      <c r="F45" t="n">
+        <v>48.2</v>
+      </c>
+      <c r="G45" t="n">
+        <v>29.1</v>
+      </c>
+      <c r="H45" t="n">
+        <v>22.1</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1297,6 +1708,15 @@
       <c r="E46" t="n">
         <v>3060</v>
       </c>
+      <c r="F46" t="n">
+        <v>48.5</v>
+      </c>
+      <c r="G46" t="n">
+        <v>29.3</v>
+      </c>
+      <c r="H46" t="n">
+        <v>22.2</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1316,6 +1736,15 @@
       <c r="E47" t="n">
         <v>2700</v>
       </c>
+      <c r="F47" t="n">
+        <v>48.7</v>
+      </c>
+      <c r="G47" t="n">
+        <v>29.6</v>
+      </c>
+      <c r="H47" t="n">
+        <v>22.3</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1335,6 +1764,15 @@
       <c r="E48" t="n">
         <v>2330</v>
       </c>
+      <c r="F48" t="n">
+        <v>48.90000000000001</v>
+      </c>
+      <c r="G48" t="n">
+        <v>29.8</v>
+      </c>
+      <c r="H48" t="n">
+        <v>22.4</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1354,6 +1792,15 @@
       <c r="E49" t="n">
         <v>1950</v>
       </c>
+      <c r="F49" t="n">
+        <v>49.2</v>
+      </c>
+      <c r="G49" t="n">
+        <v>30</v>
+      </c>
+      <c r="H49" t="n">
+        <v>22.5</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1373,6 +1820,15 @@
       <c r="E50" t="n">
         <v>2900</v>
       </c>
+      <c r="F50" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="G50" t="n">
+        <v>24.7</v>
+      </c>
+      <c r="H50" t="n">
+        <v>19.3</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1392,6 +1848,15 @@
       <c r="E51" t="n">
         <v>2200</v>
       </c>
+      <c r="F51" t="n">
+        <v>49.1</v>
+      </c>
+      <c r="G51" t="n">
+        <v>25.1</v>
+      </c>
+      <c r="H51" t="n">
+        <v>19.5</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1411,6 +1876,15 @@
       <c r="E52" t="n">
         <v>1850</v>
       </c>
+      <c r="F52" t="n">
+        <v>49.3</v>
+      </c>
+      <c r="G52" t="n">
+        <v>25.3</v>
+      </c>
+      <c r="H52" t="n">
+        <v>19.6</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1430,6 +1904,15 @@
       <c r="E53" t="n">
         <v>5150</v>
       </c>
+      <c r="F53" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="G53" t="n">
+        <v>37.9</v>
+      </c>
+      <c r="H53" t="n">
+        <v>24.7</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1449,6 +1932,15 @@
       <c r="E54" t="n">
         <v>4470</v>
       </c>
+      <c r="F54" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="G54" t="n">
+        <v>38.3</v>
+      </c>
+      <c r="H54" t="n">
+        <v>24.8</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1468,6 +1960,15 @@
       <c r="E55" t="n">
         <v>3790</v>
       </c>
+      <c r="F55" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="G55" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="H55" t="n">
+        <v>24.8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1487,6 +1988,15 @@
       <c r="E56" t="n">
         <v>3060</v>
       </c>
+      <c r="F56" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="G56" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="H56" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1506,6 +2016,15 @@
       <c r="E57" t="n">
         <v>2700</v>
       </c>
+      <c r="F57" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="G57" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="H57" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1525,6 +2044,15 @@
       <c r="E58" t="n">
         <v>2330</v>
       </c>
+      <c r="F58" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="G58" t="n">
+        <v>39.5</v>
+      </c>
+      <c r="H58" t="n">
+        <v>25.1</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1544,6 +2072,15 @@
       <c r="E59" t="n">
         <v>1950</v>
       </c>
+      <c r="F59" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="G59" t="n">
+        <v>39.8</v>
+      </c>
+      <c r="H59" t="n">
+        <v>25.2</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1563,6 +2100,15 @@
       <c r="E60" t="n">
         <v>3740</v>
       </c>
+      <c r="F60" t="n">
+        <v>39.3</v>
+      </c>
+      <c r="G60" t="n">
+        <v>24.8</v>
+      </c>
+      <c r="H60" t="n">
+        <v>19</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1582,6 +2128,15 @@
       <c r="E61" t="n">
         <v>3180</v>
       </c>
+      <c r="F61" t="n">
+        <v>39.7</v>
+      </c>
+      <c r="G61" t="n">
+        <v>25.2</v>
+      </c>
+      <c r="H61" t="n">
+        <v>19.1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1601,6 +2156,15 @@
       <c r="E62" t="n">
         <v>2580</v>
       </c>
+      <c r="F62" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="G62" t="n">
+        <v>25.6</v>
+      </c>
+      <c r="H62" t="n">
+        <v>19.2</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1620,6 +2184,15 @@
       <c r="E63" t="n">
         <v>1970</v>
       </c>
+      <c r="F63" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G63" t="n">
+        <v>26</v>
+      </c>
+      <c r="H63" t="n">
+        <v>19.3</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1639,6 +2212,15 @@
       <c r="E64" t="n">
         <v>1650</v>
       </c>
+      <c r="F64" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="G64" t="n">
+        <v>26.2</v>
+      </c>
+      <c r="H64" t="n">
+        <v>19.4</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1658,6 +2240,15 @@
       <c r="E65" t="n">
         <v>1330</v>
       </c>
+      <c r="F65" t="n">
+        <v>41</v>
+      </c>
+      <c r="G65" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="H65" t="n">
+        <v>19.6</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1677,6 +2268,15 @@
       <c r="E66" t="n">
         <v>2420</v>
       </c>
+      <c r="F66" t="n">
+        <v>40.3</v>
+      </c>
+      <c r="G66" t="n">
+        <v>21.1</v>
+      </c>
+      <c r="H66" t="n">
+        <v>16.5</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1696,6 +2296,15 @@
       <c r="E67" t="n">
         <v>2130</v>
       </c>
+      <c r="F67" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G67" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="H67" t="n">
+        <v>16.5</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1715,6 +2324,15 @@
       <c r="E68" t="n">
         <v>1850</v>
       </c>
+      <c r="F68" t="n">
+        <v>40.8</v>
+      </c>
+      <c r="G68" t="n">
+        <v>21.5</v>
+      </c>
+      <c r="H68" t="n">
+        <v>16.6</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1734,6 +2352,15 @@
       <c r="E69" t="n">
         <v>1550</v>
       </c>
+      <c r="F69" t="n">
+        <v>41</v>
+      </c>
+      <c r="G69" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="H69" t="n">
+        <v>16.7</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1753,6 +2380,15 @@
       <c r="E70" t="n">
         <v>1250</v>
       </c>
+      <c r="F70" t="n">
+        <v>41.2</v>
+      </c>
+      <c r="G70" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="H70" t="n">
+        <v>16.8</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1772,6 +2408,15 @@
       <c r="E71" t="n">
         <v>3520</v>
       </c>
+      <c r="F71" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="G71" t="n">
+        <v>30.3</v>
+      </c>
+      <c r="H71" t="n">
+        <v>19.8</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1791,6 +2436,15 @@
       <c r="E72" t="n">
         <v>2990</v>
       </c>
+      <c r="F72" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="G72" t="n">
+        <v>30.7</v>
+      </c>
+      <c r="H72" t="n">
+        <v>19.9</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1810,6 +2464,15 @@
       <c r="E73" t="n">
         <v>2430</v>
       </c>
+      <c r="F73" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="G73" t="n">
+        <v>31.1</v>
+      </c>
+      <c r="H73" t="n">
+        <v>19.9</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1829,6 +2492,15 @@
       <c r="E74" t="n">
         <v>2140</v>
       </c>
+      <c r="F74" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="G74" t="n">
+        <v>31.3</v>
+      </c>
+      <c r="H74" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1848,6 +2520,15 @@
       <c r="E75" t="n">
         <v>1850</v>
       </c>
+      <c r="F75" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="G75" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="H75" t="n">
+        <v>20.1</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1867,6 +2548,15 @@
       <c r="E76" t="n">
         <v>1560</v>
       </c>
+      <c r="F76" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="G76" t="n">
+        <v>31.7</v>
+      </c>
+      <c r="H76" t="n">
+        <v>20.2</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1886,6 +2576,15 @@
       <c r="E77" t="n">
         <v>1260</v>
       </c>
+      <c r="F77" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="G77" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="H77" t="n">
+        <v>20.3</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1905,6 +2604,15 @@
       <c r="E78" t="n">
         <v>2260</v>
       </c>
+      <c r="F78" t="n">
+        <v>31.5</v>
+      </c>
+      <c r="G78" t="n">
+        <v>26.4</v>
+      </c>
+      <c r="H78" t="n">
+        <v>18.4</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1924,6 +2632,15 @@
       <c r="E79" t="n">
         <v>1730</v>
       </c>
+      <c r="F79" t="n">
+        <v>31.9</v>
+      </c>
+      <c r="G79" t="n">
+        <v>26.8</v>
+      </c>
+      <c r="H79" t="n">
+        <v>18.5</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1943,6 +2660,15 @@
       <c r="E80" t="n">
         <v>1450</v>
       </c>
+      <c r="F80" t="n">
+        <v>32.1</v>
+      </c>
+      <c r="G80" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="H80" t="n">
+        <v>18.6</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1962,6 +2688,15 @@
       <c r="E81" t="n">
         <v>1170</v>
       </c>
+      <c r="F81" t="n">
+        <v>32.3</v>
+      </c>
+      <c r="G81" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="H81" t="n">
+        <v>18.7</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1981,6 +2716,15 @@
       <c r="E82" t="n">
         <v>2580</v>
       </c>
+      <c r="F82" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="G82" t="n">
+        <v>21.6</v>
+      </c>
+      <c r="H82" t="n">
+        <v>16.2</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -2000,6 +2744,15 @@
       <c r="E83" t="n">
         <v>2100</v>
       </c>
+      <c r="F83" t="n">
+        <v>31.8</v>
+      </c>
+      <c r="G83" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="H83" t="n">
+        <v>16.2</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -2019,6 +2772,15 @@
       <c r="E84" t="n">
         <v>1610</v>
       </c>
+      <c r="F84" t="n">
+        <v>32.2</v>
+      </c>
+      <c r="G84" t="n">
+        <v>22.3</v>
+      </c>
+      <c r="H84" t="n">
+        <v>16.4</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -2038,6 +2800,15 @@
       <c r="E85" t="n">
         <v>1350</v>
       </c>
+      <c r="F85" t="n">
+        <v>32.4</v>
+      </c>
+      <c r="G85" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="H85" t="n">
+        <v>16.5</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -2057,6 +2828,15 @@
       <c r="E86" t="n">
         <v>1090</v>
       </c>
+      <c r="F86" t="n">
+        <v>32.7</v>
+      </c>
+      <c r="G86" t="n">
+        <v>22.7</v>
+      </c>
+      <c r="H86" t="n">
+        <v>16.6</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -2076,6 +2856,15 @@
       <c r="E87" t="n">
         <v>2100</v>
       </c>
+      <c r="F87" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="G87" t="n">
+        <v>26.9</v>
+      </c>
+      <c r="H87" t="n">
+        <v>17.3</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2095,6 +2884,15 @@
       <c r="E88" t="n">
         <v>1850</v>
       </c>
+      <c r="F88" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="G88" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="H88" t="n">
+        <v>17.4</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2114,6 +2912,15 @@
       <c r="E89" t="n">
         <v>1600</v>
       </c>
+      <c r="F89" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="G89" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="H89" t="n">
+        <v>17.4</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2133,6 +2940,15 @@
       <c r="E90" t="n">
         <v>1350</v>
       </c>
+      <c r="F90" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="G90" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="H90" t="n">
+        <v>17.5</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2152,6 +2968,15 @@
       <c r="E91" t="n">
         <v>1090</v>
       </c>
+      <c r="F91" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="G91" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="H91" t="n">
+        <v>17.6</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2171,6 +2996,15 @@
       <c r="E92" t="n">
         <v>1940</v>
       </c>
+      <c r="F92" t="n">
+        <v>27.3</v>
+      </c>
+      <c r="G92" t="n">
+        <v>22.4</v>
+      </c>
+      <c r="H92" t="n">
+        <v>15.8</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2190,6 +3024,15 @@
       <c r="E93" t="n">
         <v>1710</v>
       </c>
+      <c r="F93" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="G93" t="n">
+        <v>22.6</v>
+      </c>
+      <c r="H93" t="n">
+        <v>15.8</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2209,6 +3052,15 @@
       <c r="E94" t="n">
         <v>1480</v>
       </c>
+      <c r="F94" t="n">
+        <v>27.7</v>
+      </c>
+      <c r="G94" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="H94" t="n">
+        <v>15.9</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2228,6 +3080,15 @@
       <c r="E95" t="n">
         <v>1250</v>
       </c>
+      <c r="F95" t="n">
+        <v>27.9</v>
+      </c>
+      <c r="G95" t="n">
+        <v>23</v>
+      </c>
+      <c r="H95" t="n">
+        <v>15.9</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2247,6 +3108,15 @@
       <c r="E96" t="n">
         <v>1010</v>
       </c>
+      <c r="F96" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="G96" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="H96" t="n">
+        <v>16</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2266,6 +3136,15 @@
       <c r="E97" t="n">
         <v>1770</v>
       </c>
+      <c r="F97" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="G97" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="H97" t="n">
+        <v>13.6</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2285,6 +3164,15 @@
       <c r="E98" t="n">
         <v>1360</v>
       </c>
+      <c r="F98" t="n">
+        <v>28</v>
+      </c>
+      <c r="G98" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="H98" t="n">
+        <v>13.6</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2304,6 +3192,15 @@
       <c r="E99" t="n">
         <v>1150</v>
       </c>
+      <c r="F99" t="n">
+        <v>28.2</v>
+      </c>
+      <c r="G99" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="H99" t="n">
+        <v>13.7</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2323,6 +3220,15 @@
       <c r="E100" t="n">
         <v>927</v>
       </c>
+      <c r="F100" t="n">
+        <v>28.4</v>
+      </c>
+      <c r="G100" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="H100" t="n">
+        <v>13.8</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2342,6 +3248,15 @@
       <c r="E101" t="n">
         <v>1770</v>
       </c>
+      <c r="F101" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="G101" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="H101" t="n">
+        <v>14.8</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2361,6 +3276,15 @@
       <c r="E102" t="n">
         <v>1570</v>
       </c>
+      <c r="F102" t="n">
+        <v>23</v>
+      </c>
+      <c r="G102" t="n">
+        <v>23</v>
+      </c>
+      <c r="H102" t="n">
+        <v>14.9</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2380,6 +3304,15 @@
       <c r="E103" t="n">
         <v>1360</v>
       </c>
+      <c r="F103" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="G103" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="H103" t="n">
+        <v>14.9</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2399,6 +3332,15 @@
       <c r="E104" t="n">
         <v>1150</v>
       </c>
+      <c r="F104" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G104" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="H104" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2418,6 +3360,15 @@
       <c r="E105" t="n">
         <v>927</v>
       </c>
+      <c r="F105" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="G105" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="H105" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2437,6 +3388,15 @@
       <c r="E106" t="n">
         <v>703</v>
       </c>
+      <c r="F106" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="G106" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="H106" t="n">
+        <v>15.1</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2456,6 +3416,15 @@
       <c r="E107" t="n">
         <v>1610</v>
       </c>
+      <c r="F107" t="n">
+        <v>23.2</v>
+      </c>
+      <c r="G107" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="H107" t="n">
+        <v>13.2</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2475,6 +3444,15 @@
       <c r="E108" t="n">
         <v>1430</v>
       </c>
+      <c r="F108" t="n">
+        <v>23.4</v>
+      </c>
+      <c r="G108" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="H108" t="n">
+        <v>13.2</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2494,6 +3472,15 @@
       <c r="E109" t="n">
         <v>1240</v>
       </c>
+      <c r="F109" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="G109" t="n">
+        <v>18.7</v>
+      </c>
+      <c r="H109" t="n">
+        <v>13.3</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2513,6 +3500,15 @@
       <c r="E110" t="n">
         <v>1050</v>
       </c>
+      <c r="F110" t="n">
+        <v>23.8</v>
+      </c>
+      <c r="G110" t="n">
+        <v>18.9</v>
+      </c>
+      <c r="H110" t="n">
+        <v>13.3</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2532,6 +3528,15 @@
       <c r="E111" t="n">
         <v>847</v>
       </c>
+      <c r="F111" t="n">
+        <v>24</v>
+      </c>
+      <c r="G111" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="H111" t="n">
+        <v>13.4</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2551,6 +3556,15 @@
       <c r="E112" t="n">
         <v>642</v>
       </c>
+      <c r="F112" t="n">
+        <v>24.2</v>
+      </c>
+      <c r="G112" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="H112" t="n">
+        <v>13.5</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2570,6 +3584,15 @@
       <c r="E113" t="n">
         <v>1450</v>
       </c>
+      <c r="F113" t="n">
+        <v>23.5</v>
+      </c>
+      <c r="G113" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="H113" t="n">
+        <v>10.9</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2589,6 +3612,15 @@
       <c r="E114" t="n">
         <v>1120</v>
       </c>
+      <c r="F114" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="G114" t="n">
+        <v>14.2</v>
+      </c>
+      <c r="H114" t="n">
+        <v>10.9</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2608,6 +3640,15 @@
       <c r="E115" t="n">
         <v>945</v>
       </c>
+      <c r="F115" t="n">
+        <v>24.1</v>
+      </c>
+      <c r="G115" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="H115" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2627,6 +3668,15 @@
       <c r="E116" t="n">
         <v>766</v>
       </c>
+      <c r="F116" t="n">
+        <v>24.3</v>
+      </c>
+      <c r="G116" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="H116" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2646,6 +3696,15 @@
       <c r="E117" t="n">
         <v>582</v>
       </c>
+      <c r="F117" t="n">
+        <v>24.5</v>
+      </c>
+      <c r="G117" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="H117" t="n">
+        <v>11.1</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2665,6 +3724,15 @@
       <c r="E118" t="n">
         <v>1450</v>
       </c>
+      <c r="F118" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G118" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="H118" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2684,6 +3752,15 @@
       <c r="E119" t="n">
         <v>1120</v>
       </c>
+      <c r="F119" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="G119" t="n">
+        <v>19.1</v>
+      </c>
+      <c r="H119" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2703,6 +3780,15 @@
       <c r="E120" t="n">
         <v>945</v>
       </c>
+      <c r="F120" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="G120" t="n">
+        <v>19.3</v>
+      </c>
+      <c r="H120" t="n">
+        <v>12.4</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2722,6 +3808,15 @@
       <c r="E121" t="n">
         <v>766</v>
       </c>
+      <c r="F121" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G121" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="H121" t="n">
+        <v>12.5</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2741,6 +3836,15 @@
       <c r="E122" t="n">
         <v>582</v>
       </c>
+      <c r="F122" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="G122" t="n">
+        <v>19.8</v>
+      </c>
+      <c r="H122" t="n">
+        <v>12.6</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2760,6 +3864,15 @@
       <c r="E123" t="n">
         <v>998</v>
       </c>
+      <c r="F123" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G123" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="H123" t="n">
+        <v>10.7</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2779,6 +3892,15 @@
       <c r="E124" t="n">
         <v>844</v>
       </c>
+      <c r="F124" t="n">
+        <v>19.7</v>
+      </c>
+      <c r="G124" t="n">
+        <v>14.8</v>
+      </c>
+      <c r="H124" t="n">
+        <v>10.7</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2798,6 +3920,15 @@
       <c r="E125" t="n">
         <v>685</v>
       </c>
+      <c r="F125" t="n">
+        <v>19.9</v>
+      </c>
+      <c r="G125" t="n">
+        <v>15</v>
+      </c>
+      <c r="H125" t="n">
+        <v>10.8</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2817,6 +3948,15 @@
       <c r="E126" t="n">
         <v>521</v>
       </c>
+      <c r="F126" t="n">
+        <v>20.1</v>
+      </c>
+      <c r="G126" t="n">
+        <v>15.2</v>
+      </c>
+      <c r="H126" t="n">
+        <v>10.9</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2836,6 +3976,15 @@
       <c r="E127" t="n">
         <v>605</v>
       </c>
+      <c r="F127" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="G127" t="n">
+        <v>10.5</v>
+      </c>
+      <c r="H127" t="n">
+        <v>8.23</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2855,6 +4004,15 @@
       <c r="E128" t="n">
         <v>461</v>
       </c>
+      <c r="F128" t="n">
+        <v>20.4</v>
+      </c>
+      <c r="G128" t="n">
+        <v>10.7</v>
+      </c>
+      <c r="H128" t="n">
+        <v>8.31</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -2874,6 +4032,15 @@
       <c r="E129" t="n">
         <v>877</v>
       </c>
+      <c r="F129" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="G129" t="n">
+        <v>15.1</v>
+      </c>
+      <c r="H129" t="n">
+        <v>9.890000000000001</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -2893,6 +4060,15 @@
       <c r="E130" t="n">
         <v>744</v>
       </c>
+      <c r="F130" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="G130" t="n">
+        <v>15.3</v>
+      </c>
+      <c r="H130" t="n">
+        <v>9.9</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2912,6 +4088,15 @@
       <c r="E131" t="n">
         <v>605</v>
       </c>
+      <c r="F131" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G131" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="H131" t="n">
+        <v>9.93</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -2931,6 +4116,15 @@
       <c r="E132" t="n">
         <v>461</v>
       </c>
+      <c r="F132" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="G132" t="n">
+        <v>15.7</v>
+      </c>
+      <c r="H132" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2950,6 +4144,15 @@
       <c r="E133" t="n">
         <v>313</v>
       </c>
+      <c r="F133" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="G133" t="n">
+        <v>15.9</v>
+      </c>
+      <c r="H133" t="n">
+        <v>10.1</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2969,6 +4172,15 @@
       <c r="E134" t="n">
         <v>524</v>
       </c>
+      <c r="F134" t="n">
+        <v>15.8</v>
+      </c>
+      <c r="G134" t="n">
+        <v>11</v>
+      </c>
+      <c r="H134" t="n">
+        <v>8.119999999999999</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2988,6 +4200,15 @@
       <c r="E135" t="n">
         <v>401</v>
       </c>
+      <c r="F135" t="n">
+        <v>16</v>
+      </c>
+      <c r="G135" t="n">
+        <v>11.2</v>
+      </c>
+      <c r="H135" t="n">
+        <v>8.18</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -3007,6 +4228,15 @@
       <c r="E136" t="n">
         <v>273</v>
       </c>
+      <c r="F136" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="G136" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H136" t="n">
+        <v>8.27</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -3026,6 +4256,15 @@
       <c r="E137" t="n">
         <v>525</v>
       </c>
+      <c r="F137" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G137" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="H137" t="n">
+        <v>8.68</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -3045,6 +4284,15 @@
       <c r="E138" t="n">
         <v>401</v>
       </c>
+      <c r="F138" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G138" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="H138" t="n">
+        <v>8.73</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -3064,6 +4312,15 @@
       <c r="E139" t="n">
         <v>273</v>
       </c>
+      <c r="F139" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="G139" t="n">
+        <v>13.9</v>
+      </c>
+      <c r="H139" t="n">
+        <v>8.82</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -3083,6 +4340,15 @@
       <c r="E140" t="n">
         <v>444</v>
       </c>
+      <c r="F140" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="G140" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="H140" t="n">
+        <v>7.42</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -3102,6 +4368,15 @@
       <c r="E141" t="n">
         <v>340</v>
       </c>
+      <c r="F141" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="G141" t="n">
+        <v>11.6</v>
+      </c>
+      <c r="H141" t="n">
+        <v>7.45</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -3121,6 +4396,15 @@
       <c r="E142" t="n">
         <v>287</v>
       </c>
+      <c r="F142" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="G142" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="H142" t="n">
+        <v>7.48</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -3140,6 +4424,15 @@
       <c r="E143" t="n">
         <v>232</v>
       </c>
+      <c r="F143" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="G143" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="H143" t="n">
+        <v>7.52</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3159,6 +4452,15 @@
       <c r="E144" t="n">
         <v>364</v>
       </c>
+      <c r="F144" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G144" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="H144" t="n">
+        <v>6.19</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3178,6 +4480,15 @@
       <c r="E145" t="n">
         <v>280</v>
       </c>
+      <c r="F145" t="n">
+        <v>9.58</v>
+      </c>
+      <c r="G145" t="n">
+        <v>9.58</v>
+      </c>
+      <c r="H145" t="n">
+        <v>6.2</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3197,6 +4508,15 @@
       <c r="E146" t="n">
         <v>192</v>
       </c>
+      <c r="F146" t="n">
+        <v>9.790000000000001</v>
+      </c>
+      <c r="G146" t="n">
+        <v>9.790000000000001</v>
+      </c>
+      <c r="H146" t="n">
+        <v>6.25</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3216,6 +4536,15 @@
       <c r="E147" t="n">
         <v>282</v>
       </c>
+      <c r="F147" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="G147" t="n">
+        <v>7.37</v>
+      </c>
+      <c r="H147" t="n">
+        <v>4.98</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3235,6 +4564,15 @@
       <c r="E148" t="n">
         <v>219</v>
       </c>
+      <c r="F148" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="G148" t="n">
+        <v>7.54</v>
+      </c>
+      <c r="H148" t="n">
+        <v>4.94</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3254,6 +4592,15 @@
       <c r="E149" t="n">
         <v>151</v>
       </c>
+      <c r="F149" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="G149" t="n">
+        <v>7.73</v>
+      </c>
+      <c r="H149" t="n">
+        <v>4.97</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3272,6 +4619,15 @@
       </c>
       <c r="E150" t="n">
         <v>111</v>
+      </c>
+      <c r="F150" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="G150" t="n">
+        <v>5.72</v>
+      </c>
+      <c r="H150" t="n">
+        <v>3.72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>